<commit_message>
add notes to compare script
</commit_message>
<xml_diff>
--- a/dune-results/dr_comparison_2026.xlsx
+++ b/dune-results/dr_comparison_2026.xlsx
@@ -3,11 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Our Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Soter Data" sheetId="1" r:id="rId1"/>
     <sheet name="Spark" sheetId="2" r:id="rId2"/>
     <sheet name="Amatsu" sheetId="3" r:id="rId3"/>
-    <sheet name="Diff Ours-Spark" sheetId="4" r:id="rId4"/>
-    <sheet name="Diff Ours-Amatsu" sheetId="5" r:id="rId5"/>
+    <sheet name="Diff Soter-Spark" sheetId="4" r:id="rId4"/>
+    <sheet name="Diff Soter-Amatsu" sheetId="5" r:id="rId5"/>
     <sheet name="Diff Spark-Amatsu" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:H76"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -411,6 +411,7 @@
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
     <col min="6" max="6" width="13.83203125" customWidth="1"/>
     <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -435,6 +436,9 @@
       <c r="G1" t="str">
         <v>total</v>
       </c>
+      <c r="H1" t="str">
+        <v>notes</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -458,6 +462,9 @@
       <c r="G2">
         <v>0</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -481,6 +488,9 @@
       <c r="G3">
         <v>0</v>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -504,6 +514,9 @@
       <c r="G4">
         <v>62.45</v>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -527,6 +540,9 @@
       <c r="G5">
         <v>367746.75</v>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -550,6 +566,9 @@
       <c r="G6">
         <v>1786.39</v>
       </c>
+      <c r="H6" t="str">
+        <v>Chronicle farm — not tracked by Spark/BA.</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -573,6 +592,9 @@
       <c r="G7">
         <v>183.39</v>
       </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -596,6 +618,9 @@
       <c r="G8">
         <v>476.01</v>
       </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -619,6 +644,9 @@
       <c r="G9">
         <v>14506.79</v>
       </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -642,6 +670,9 @@
       <c r="G10">
         <v>443531.96</v>
       </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -665,6 +696,9 @@
       <c r="G11">
         <v>29341.39</v>
       </c>
+      <c r="H11" t="str">
+        <v>Chronicle farm — not tracked by Spark/BA.</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -688,6 +722,9 @@
       <c r="G12">
         <v>38223.42</v>
       </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -711,6 +748,9 @@
       <c r="G13">
         <v>66951.14</v>
       </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -734,6 +774,9 @@
       <c r="G14">
         <v>0</v>
       </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -757,6 +800,9 @@
       <c r="G15">
         <v>0</v>
       </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -780,539 +826,611 @@
       <c r="G16">
         <v>0</v>
       </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>127</v>
-      </c>
-      <c r="B17">
-        <v>3037.15</v>
-      </c>
-      <c r="C17">
-        <v>2639.18</v>
-      </c>
-      <c r="D17">
-        <v>2167.44</v>
-      </c>
-      <c r="E17">
-        <v>1447.5</v>
-      </c>
-      <c r="F17">
-        <v>730.93</v>
+        <v>126</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
       </c>
       <c r="G17">
-        <v>10022.2</v>
+        <v>0</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Subproxy holdings, no DR applied. Handled in Supply Side MSC.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B18">
-        <v>826847.7</v>
+        <v>3037.15</v>
       </c>
       <c r="C18">
-        <v>837591.56</v>
+        <v>2639.18</v>
       </c>
       <c r="D18">
-        <v>1199709.46</v>
+        <v>2167.44</v>
       </c>
       <c r="E18">
-        <v>1321957.96</v>
+        <v>1447.5</v>
       </c>
       <c r="F18">
-        <v>1461137.84</v>
+        <v>730.93</v>
       </c>
       <c r="G18">
-        <v>5647244.52</v>
+        <v>10022.2</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Spark untagged Savings, had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B19">
-        <v>1.03</v>
+        <v>826847.7</v>
       </c>
       <c r="C19">
-        <v>0.52</v>
+        <v>837591.56</v>
       </c>
       <c r="D19">
-        <v>0.67</v>
+        <v>1199709.46</v>
       </c>
       <c r="E19">
-        <v>0.77</v>
+        <v>1321957.96</v>
       </c>
       <c r="F19">
-        <v>1.13</v>
+        <v>1461137.84</v>
       </c>
       <c r="G19">
-        <v>4.12</v>
+        <v>5647244.52</v>
+      </c>
+      <c r="H19" t="str">
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>170</v>
+        <v>129</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>1.03</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>0.67</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>1.13</v>
       </c>
       <c r="G20">
-        <v>0</v>
+        <v>4.12</v>
+      </c>
+      <c r="H20" t="str">
+        <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>171</v>
-      </c>
-      <c r="B21">
-        <v>0</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>0</v>
-      </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
+        <v>130</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
       </c>
       <c r="G21">
         <v>0</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Found in Spark datasets only, no onchain events.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="B22">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="C22">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="D22">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E22">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="F22">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>0.05</v>
+        <v>0</v>
+      </c>
+      <c r="H22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="B23">
-        <v>21333.38</v>
+        <v>0</v>
       </c>
       <c r="C23">
-        <v>13278.93</v>
+        <v>0</v>
       </c>
       <c r="D23">
-        <v>11113.76</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>9912.97</v>
+        <v>0</v>
       </c>
       <c r="F23">
-        <v>11847.6</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>67486.64</v>
+        <v>0</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B24">
-        <v>467.21</v>
+        <v>0.01</v>
       </c>
       <c r="C24">
-        <v>638.59</v>
+        <v>0.01</v>
       </c>
       <c r="D24">
-        <v>1188.8</v>
+        <v>0.01</v>
       </c>
       <c r="E24">
-        <v>1386.57</v>
+        <v>0.01</v>
       </c>
       <c r="F24">
-        <v>1241.16</v>
+        <v>0.01</v>
       </c>
       <c r="G24">
-        <v>4922.33</v>
+        <v>0.05</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="B25">
-        <v>475.33</v>
+        <v>21333.38</v>
       </c>
       <c r="C25">
-        <v>108.27</v>
+        <v>13278.93</v>
       </c>
       <c r="D25">
-        <v>7201.39</v>
+        <v>11113.76</v>
       </c>
       <c r="E25">
-        <v>14582.19</v>
+        <v>9912.97</v>
       </c>
       <c r="F25">
-        <v>11608.11</v>
+        <v>11847.6</v>
       </c>
       <c r="G25">
-        <v>33975.29</v>
+        <v>67486.64</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B26">
-        <v>10427.71</v>
+        <v>467.21</v>
       </c>
       <c r="C26">
-        <v>5314.13</v>
+        <v>638.59</v>
       </c>
       <c r="D26">
-        <v>4209.1</v>
+        <v>1188.8</v>
       </c>
       <c r="E26">
-        <v>2912.07</v>
+        <v>1386.57</v>
       </c>
       <c r="F26">
-        <v>2740.89</v>
+        <v>1241.16</v>
       </c>
       <c r="G26">
-        <v>25603.9</v>
+        <v>4922.33</v>
+      </c>
+      <c r="H26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B27">
-        <v>3326.25</v>
+        <v>475.33</v>
       </c>
       <c r="C27">
-        <v>5352.96</v>
+        <v>108.27</v>
       </c>
       <c r="D27">
-        <v>8218.73</v>
+        <v>7201.39</v>
       </c>
       <c r="E27">
-        <v>12123.38</v>
+        <v>14582.19</v>
       </c>
       <c r="F27">
-        <v>23241.91</v>
+        <v>11608.11</v>
       </c>
       <c r="G27">
-        <v>52263.23</v>
+        <v>33975.29</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B28">
-        <v>22700.54</v>
+        <v>10427.71</v>
       </c>
       <c r="C28">
-        <v>16725.41</v>
+        <v>5314.13</v>
       </c>
       <c r="D28">
-        <v>19342.47</v>
+        <v>4209.1</v>
       </c>
       <c r="E28">
-        <v>15097.77</v>
+        <v>2912.07</v>
       </c>
       <c r="F28">
-        <v>10576.24</v>
+        <v>2740.89</v>
       </c>
       <c r="G28">
-        <v>84442.43</v>
+        <v>25603.9</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="29">
       <c r="A29">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B29">
-        <v>1.99</v>
+        <v>3326.25</v>
       </c>
       <c r="C29">
-        <v>1.7</v>
+        <v>5352.96</v>
       </c>
       <c r="D29">
-        <v>1.88</v>
+        <v>8218.73</v>
       </c>
       <c r="E29">
-        <v>1.72</v>
+        <v>12123.38</v>
       </c>
       <c r="F29">
-        <v>1.75</v>
+        <v>23241.91</v>
       </c>
       <c r="G29">
-        <v>9.04</v>
+        <v>52263.23</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B30">
-        <v>1554.29</v>
+        <v>22700.54</v>
       </c>
       <c r="C30">
-        <v>669.49</v>
+        <v>16725.41</v>
       </c>
       <c r="D30">
-        <v>3049.96</v>
+        <v>19342.47</v>
       </c>
       <c r="E30">
-        <v>1990.3</v>
+        <v>15097.77</v>
       </c>
       <c r="F30">
-        <v>1235.01</v>
+        <v>10576.24</v>
       </c>
       <c r="G30">
-        <v>8499.05</v>
+        <v>84442.43</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B31">
-        <v>0.01</v>
+        <v>1.99</v>
       </c>
       <c r="C31">
-        <v>0.09</v>
+        <v>1.7</v>
       </c>
       <c r="D31">
-        <v>0.1</v>
+        <v>1.88</v>
       </c>
       <c r="E31">
-        <v>0.1</v>
+        <v>1.72</v>
       </c>
       <c r="F31">
-        <v>0.1</v>
+        <v>1.75</v>
       </c>
       <c r="G31">
-        <v>0.4</v>
+        <v>9.04</v>
+      </c>
+      <c r="H31" t="str">
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B32">
-        <v>6824.99</v>
+        <v>1554.29</v>
       </c>
       <c r="C32">
-        <v>6314.15</v>
+        <v>669.49</v>
       </c>
       <c r="D32">
-        <v>5576.07</v>
+        <v>3049.96</v>
       </c>
       <c r="E32">
-        <v>8508.93</v>
+        <v>1990.3</v>
       </c>
       <c r="F32">
-        <v>10729.88</v>
+        <v>1235.01</v>
       </c>
       <c r="G32">
-        <v>37954.02</v>
+        <v>8499.05</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B33">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="C33">
-        <v>0.02</v>
+        <v>0.09</v>
       </c>
       <c r="D33">
-        <v>0.02</v>
+        <v>0.1</v>
       </c>
       <c r="E33">
-        <v>0.02</v>
+        <v>0.1</v>
       </c>
       <c r="F33">
-        <v>0.02</v>
+        <v>0.1</v>
       </c>
       <c r="G33">
-        <v>0.1</v>
+        <v>0.4</v>
+      </c>
+      <c r="H33" t="str">
+        <v/>
       </c>
     </row>
     <row r="34">
       <c r="A34">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B34">
-        <v>1.96</v>
+        <v>6824.99</v>
       </c>
       <c r="C34">
-        <v>0.65</v>
+        <v>6314.15</v>
       </c>
       <c r="D34">
-        <v>5.79</v>
+        <v>5576.07</v>
       </c>
       <c r="E34">
-        <v>32.59</v>
+        <v>8508.93</v>
       </c>
       <c r="F34">
-        <v>91.6</v>
+        <v>10729.88</v>
       </c>
       <c r="G34">
-        <v>132.59</v>
+        <v>37954.02</v>
+      </c>
+      <c r="H34" t="str">
+        <v>stUSDS. Amatsu/BA applied DR in Jan./Feb. then switched to 0.1% after. s/b 0.1% always applied.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B35">
-        <v>28.54</v>
+        <v>0.02</v>
       </c>
       <c r="C35">
-        <v>32.89</v>
+        <v>0.02</v>
       </c>
       <c r="D35">
-        <v>42.56</v>
+        <v>0.02</v>
       </c>
       <c r="E35">
-        <v>39.75</v>
+        <v>0.02</v>
       </c>
       <c r="F35">
-        <v>33.27</v>
+        <v>0.02</v>
       </c>
       <c r="G35">
-        <v>177.01</v>
+        <v>0.1</v>
+      </c>
+      <c r="H35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>204</v>
-      </c>
-      <c r="B36" t="str">
-        <v/>
+        <v>200</v>
+      </c>
+      <c r="B36">
+        <v>1.96</v>
       </c>
       <c r="C36">
-        <v>1.61</v>
+        <v>0.65</v>
       </c>
       <c r="D36">
-        <v>16.91</v>
+        <v>5.79</v>
       </c>
       <c r="E36">
-        <v>34.05</v>
+        <v>32.59</v>
       </c>
       <c r="F36">
-        <v>30.45</v>
+        <v>91.6</v>
       </c>
       <c r="G36">
-        <v>83.02</v>
+        <v>132.59</v>
+      </c>
+      <c r="H36" t="str">
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B37">
-        <v>0</v>
+        <v>28.54</v>
       </c>
       <c r="C37">
-        <v>0.02</v>
+        <v>32.89</v>
       </c>
       <c r="D37">
-        <v>0.2</v>
+        <v>42.56</v>
       </c>
       <c r="E37">
-        <v>0.21</v>
+        <v>39.75</v>
       </c>
       <c r="F37">
-        <v>0.21</v>
+        <v>33.27</v>
       </c>
       <c r="G37">
-        <v>0.64</v>
+        <v>177.01</v>
+      </c>
+      <c r="H37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B38" t="str">
         <v/>
       </c>
-      <c r="C38" t="str">
-        <v/>
-      </c>
-      <c r="D38" t="str">
-        <v/>
-      </c>
-      <c r="E38" t="str">
-        <v/>
+      <c r="C38">
+        <v>1.61</v>
+      </c>
+      <c r="D38">
+        <v>16.91</v>
+      </c>
+      <c r="E38">
+        <v>34.05</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>30.45</v>
       </c>
       <c r="G38">
-        <v>0</v>
+        <v>83.02</v>
+      </c>
+      <c r="H38" t="str">
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39">
-        <v>214</v>
-      </c>
-      <c r="B39" t="str">
-        <v/>
-      </c>
-      <c r="C39" t="str">
-        <v/>
-      </c>
-      <c r="D39" t="str">
-        <v/>
-      </c>
-      <c r="E39" t="str">
-        <v/>
+        <v>205</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
+      </c>
+      <c r="C39">
+        <v>0.02</v>
+      </c>
+      <c r="D39">
+        <v>0.2</v>
+      </c>
+      <c r="E39">
+        <v>0.21</v>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="G39">
-        <v>0</v>
+        <v>0.64</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="B40" t="str">
         <v/>
@@ -1320,22 +1438,25 @@
       <c r="C40" t="str">
         <v/>
       </c>
-      <c r="D40">
-        <v>86.77</v>
-      </c>
-      <c r="E40">
-        <v>151.21</v>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v/>
       </c>
       <c r="F40">
-        <v>189.04</v>
+        <v>0</v>
       </c>
       <c r="G40">
-        <v>427.02</v>
+        <v>0</v>
+      </c>
+      <c r="H40" t="str">
+        <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B41" t="str">
         <v/>
@@ -1346,19 +1467,22 @@
       <c r="D41" t="str">
         <v/>
       </c>
-      <c r="E41">
-        <v>14.26</v>
-      </c>
-      <c r="F41" t="str">
-        <v/>
+      <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41">
+        <v>0</v>
       </c>
       <c r="G41">
-        <v>14.26</v>
+        <v>0</v>
+      </c>
+      <c r="H41" t="str">
+        <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="B42" t="str">
         <v/>
@@ -1366,22 +1490,25 @@
       <c r="C42" t="str">
         <v/>
       </c>
-      <c r="D42" t="str">
-        <v/>
-      </c>
-      <c r="E42" t="str">
-        <v/>
+      <c r="D42">
+        <v>86.77</v>
+      </c>
+      <c r="E42">
+        <v>151.21</v>
       </c>
       <c r="F42">
-        <v>0</v>
+        <v>189.04</v>
       </c>
       <c r="G42">
-        <v>0</v>
+        <v>427.02</v>
+      </c>
+      <c r="H42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B43" t="str">
         <v/>
@@ -1392,235 +1519,265 @@
       <c r="D43" t="str">
         <v/>
       </c>
-      <c r="E43" t="str">
-        <v/>
-      </c>
-      <c r="F43">
-        <v>4582.17</v>
+      <c r="E43">
+        <v>14.26</v>
+      </c>
+      <c r="F43" t="str">
+        <v/>
       </c>
       <c r="G43">
-        <v>4582.17</v>
+        <v>14.26</v>
+      </c>
+      <c r="H43" t="str">
+        <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44">
-        <v>303</v>
-      </c>
-      <c r="B44">
-        <v>0</v>
-      </c>
-      <c r="C44">
-        <v>0</v>
-      </c>
-      <c r="D44">
-        <v>0</v>
-      </c>
-      <c r="E44">
-        <v>0</v>
+        <v>223</v>
+      </c>
+      <c r="B44" t="str">
+        <v/>
+      </c>
+      <c r="C44" t="str">
+        <v/>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v/>
       </c>
       <c r="F44">
         <v>0</v>
       </c>
       <c r="G44">
         <v>0</v>
+      </c>
+      <c r="H44" t="str">
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>555</v>
-      </c>
-      <c r="B45">
-        <v>0</v>
-      </c>
-      <c r="C45">
-        <v>0</v>
-      </c>
-      <c r="D45">
-        <v>0</v>
-      </c>
-      <c r="E45">
-        <v>0</v>
+        <v>224</v>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v/>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>4582.17</v>
       </c>
       <c r="G45">
-        <v>0</v>
+        <v>4582.17</v>
+      </c>
+      <c r="H45" t="str">
+        <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46">
-        <v>1001</v>
+        <v>303</v>
       </c>
       <c r="B46">
-        <v>2254.8</v>
+        <v>0</v>
       </c>
       <c r="C46">
-        <v>1601.44</v>
+        <v>0</v>
       </c>
       <c r="D46">
-        <v>1655.49</v>
+        <v>0</v>
       </c>
       <c r="E46">
-        <v>1433.94</v>
+        <v>0</v>
       </c>
       <c r="F46">
-        <v>912.57</v>
+        <v>0</v>
       </c>
       <c r="G46">
-        <v>7858.24</v>
+        <v>0</v>
+      </c>
+      <c r="H46" t="str">
+        <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>1002</v>
+        <v>555</v>
       </c>
       <c r="B47">
-        <v>1969.51</v>
+        <v>0</v>
       </c>
       <c r="C47">
-        <v>2970.51</v>
+        <v>0</v>
       </c>
       <c r="D47">
-        <v>29195.53</v>
+        <v>0</v>
       </c>
       <c r="E47">
-        <v>28955.22</v>
+        <v>0</v>
       </c>
       <c r="F47">
-        <v>33175.15</v>
+        <v>0</v>
       </c>
       <c r="G47">
-        <v>96265.92</v>
+        <v>0</v>
+      </c>
+      <c r="H47" t="str">
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>1004</v>
+        <v>1001</v>
       </c>
       <c r="B48">
-        <v>0.01</v>
+        <v>2254.8</v>
       </c>
       <c r="C48">
-        <v>0</v>
+        <v>1601.44</v>
       </c>
       <c r="D48">
-        <v>0.01</v>
+        <v>1655.49</v>
       </c>
       <c r="E48">
-        <v>0.01</v>
+        <v>1433.94</v>
       </c>
       <c r="F48">
-        <v>0.01</v>
+        <v>912.57</v>
       </c>
       <c r="G48">
-        <v>0.04</v>
+        <v>7858.24</v>
+      </c>
+      <c r="H48" t="str">
+        <v>Feb. and Mar. had no DR by Amatsu.</v>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>1007</v>
+        <v>1002</v>
       </c>
       <c r="B49">
-        <v>10082.51</v>
+        <v>1969.51</v>
       </c>
       <c r="C49">
-        <v>13745.06</v>
+        <v>2970.51</v>
       </c>
       <c r="D49">
-        <v>15859.43</v>
+        <v>29195.53</v>
       </c>
       <c r="E49">
-        <v>14112.17</v>
+        <v>28955.22</v>
       </c>
       <c r="F49">
-        <v>10762.39</v>
+        <v>33175.15</v>
       </c>
       <c r="G49">
-        <v>64561.56</v>
+        <v>96265.92</v>
+      </c>
+      <c r="H49" t="str">
+        <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>1015</v>
-      </c>
-      <c r="B50">
-        <v>0</v>
-      </c>
-      <c r="C50">
-        <v>0</v>
-      </c>
-      <c r="D50">
-        <v>0</v>
-      </c>
-      <c r="E50">
-        <v>0</v>
-      </c>
-      <c r="F50">
-        <v>0</v>
+        <v>1003</v>
+      </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
+      <c r="C50" t="str">
+        <v/>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
+      <c r="F50" t="str">
+        <v/>
       </c>
       <c r="G50">
         <v>0</v>
+      </c>
+      <c r="H50" t="str">
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>1016</v>
+        <v>1004</v>
       </c>
       <c r="B51">
-        <v>1201.05</v>
+        <v>0.01</v>
       </c>
       <c r="C51">
-        <v>167.54</v>
+        <v>0</v>
       </c>
       <c r="D51">
-        <v>8.98</v>
+        <v>0.01</v>
       </c>
       <c r="E51">
-        <v>0.59</v>
-      </c>
-      <c r="F51" t="str">
-        <v/>
+        <v>0.01</v>
+      </c>
+      <c r="F51">
+        <v>0.01</v>
       </c>
       <c r="G51">
-        <v>1378.16</v>
+        <v>0.04</v>
+      </c>
+      <c r="H51" t="str">
+        <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52">
-        <v>1017</v>
+        <v>1007</v>
       </c>
       <c r="B52">
-        <v>215.45</v>
+        <v>10082.51</v>
       </c>
       <c r="C52">
-        <v>140.34</v>
+        <v>13745.06</v>
       </c>
       <c r="D52">
-        <v>148.1</v>
+        <v>15859.43</v>
       </c>
       <c r="E52">
-        <v>85.99</v>
+        <v>14112.17</v>
       </c>
       <c r="F52">
-        <v>3.52</v>
+        <v>10762.39</v>
       </c>
       <c r="G52">
-        <v>593.4</v>
+        <v>64561.56</v>
+      </c>
+      <c r="H52" t="str">
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53">
-        <v>2000</v>
-      </c>
-      <c r="B53" t="str">
-        <v/>
-      </c>
-      <c r="C53" t="str">
-        <v/>
-      </c>
-      <c r="D53" t="str">
-        <v/>
+        <v>1015</v>
+      </c>
+      <c r="B53">
+        <v>0</v>
+      </c>
+      <c r="C53">
+        <v>0</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -1630,57 +1787,66 @@
       </c>
       <c r="G53">
         <v>0</v>
+      </c>
+      <c r="H53" t="str">
+        <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54">
-        <v>2001</v>
-      </c>
-      <c r="B54" t="str">
-        <v/>
+        <v>1016</v>
+      </c>
+      <c r="B54">
+        <v>1201.05</v>
       </c>
       <c r="C54">
-        <v>0</v>
+        <v>167.54</v>
       </c>
       <c r="D54">
-        <v>0</v>
+        <v>8.98</v>
       </c>
       <c r="E54">
-        <v>82.24</v>
-      </c>
-      <c r="F54">
-        <v>8467.99</v>
+        <v>0.59</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
       </c>
       <c r="G54">
-        <v>8550.23</v>
+        <v>1378.16</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Amatsu included DR for sUSDC, sUSDS, SKY, while onchain, only events for SKY can be found. unknown which balances or events to use for sUSDC and sUSDS.</v>
       </c>
     </row>
     <row r="55">
       <c r="A55">
-        <v>2002</v>
-      </c>
-      <c r="B55" t="str">
-        <v/>
-      </c>
-      <c r="C55" t="str">
-        <v/>
+        <v>1017</v>
+      </c>
+      <c r="B55">
+        <v>215.45</v>
+      </c>
+      <c r="C55">
+        <v>140.34</v>
       </c>
       <c r="D55">
-        <v>174574.28</v>
+        <v>148.1</v>
       </c>
       <c r="E55">
-        <v>116737.37</v>
+        <v>85.99</v>
       </c>
       <c r="F55">
-        <v>0</v>
+        <v>3.52</v>
       </c>
       <c r="G55">
-        <v>291311.65</v>
+        <v>593.4</v>
+      </c>
+      <c r="H55" t="str">
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56">
-        <v>2003</v>
+        <v>2000</v>
       </c>
       <c r="B56" t="str">
         <v/>
@@ -1699,34 +1865,40 @@
       </c>
       <c r="G56">
         <v>0</v>
+      </c>
+      <c r="H56" t="str">
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57">
-        <v>2005</v>
+        <v>2001</v>
       </c>
       <c r="B57" t="str">
         <v/>
       </c>
-      <c r="C57" t="str">
-        <v/>
+      <c r="C57">
+        <v>0</v>
       </c>
       <c r="D57">
-        <v>17144.97</v>
+        <v>0</v>
       </c>
       <c r="E57">
-        <v>8259.88</v>
-      </c>
-      <c r="F57" t="str">
-        <v/>
+        <v>82.24</v>
+      </c>
+      <c r="F57">
+        <v>8467.99</v>
       </c>
       <c r="G57">
-        <v>25404.85</v>
+        <v>8550.23</v>
+      </c>
+      <c r="H57" t="str">
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58">
-        <v>2008</v>
+        <v>2002</v>
       </c>
       <c r="B58" t="str">
         <v/>
@@ -1734,22 +1906,25 @@
       <c r="C58" t="str">
         <v/>
       </c>
-      <c r="D58" t="str">
-        <v/>
-      </c>
-      <c r="E58" t="str">
-        <v/>
+      <c r="D58">
+        <v>174574.28</v>
+      </c>
+      <c r="E58">
+        <v>116737.37</v>
       </c>
       <c r="F58">
-        <v>12035.78</v>
+        <v>0</v>
       </c>
       <c r="G58">
-        <v>12035.78</v>
+        <v>291311.65</v>
+      </c>
+      <c r="H58" t="str">
+        <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59">
-        <v>2222</v>
+        <v>2003</v>
       </c>
       <c r="B59" t="str">
         <v/>
@@ -1761,18 +1936,21 @@
         <v/>
       </c>
       <c r="E59">
-        <v>10.68</v>
+        <v>0</v>
       </c>
       <c r="F59">
-        <v>14.75</v>
+        <v>0</v>
       </c>
       <c r="G59">
-        <v>25.43</v>
+        <v>0</v>
+      </c>
+      <c r="H59" t="str">
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60">
-        <v>3000</v>
+        <v>2005</v>
       </c>
       <c r="B60" t="str">
         <v/>
@@ -1780,22 +1958,25 @@
       <c r="C60" t="str">
         <v/>
       </c>
-      <c r="D60" t="str">
-        <v/>
+      <c r="D60">
+        <v>17144.97</v>
       </c>
       <c r="E60">
-        <v>0</v>
-      </c>
-      <c r="F60">
-        <v>0</v>
+        <v>8259.88</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
       </c>
       <c r="G60">
-        <v>0</v>
+        <v>25404.85</v>
+      </c>
+      <c r="H60" t="str">
+        <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61">
-        <v>3001</v>
+        <v>2008</v>
       </c>
       <c r="B61" t="str">
         <v/>
@@ -1810,38 +1991,44 @@
         <v/>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>12035.78</v>
       </c>
       <c r="G61">
-        <v>0</v>
+        <v>12035.78</v>
+      </c>
+      <c r="H61" t="str">
+        <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62">
-        <v>3333</v>
-      </c>
-      <c r="B62">
-        <v>0.71</v>
-      </c>
-      <c r="C62">
-        <v>0.41</v>
-      </c>
-      <c r="D62">
-        <v>0.48</v>
+        <v>2222</v>
+      </c>
+      <c r="B62" t="str">
+        <v/>
+      </c>
+      <c r="C62" t="str">
+        <v/>
+      </c>
+      <c r="D62" t="str">
+        <v/>
       </c>
       <c r="E62">
-        <v>0.49</v>
+        <v>10.68</v>
       </c>
       <c r="F62">
-        <v>0.48</v>
+        <v>14.75</v>
       </c>
       <c r="G62">
-        <v>2.57</v>
+        <v>25.43</v>
+      </c>
+      <c r="H62" t="str">
+        <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63">
-        <v>4011</v>
+        <v>3000</v>
       </c>
       <c r="B63" t="str">
         <v/>
@@ -1852,19 +2039,22 @@
       <c r="D63" t="str">
         <v/>
       </c>
-      <c r="E63" t="str">
-        <v/>
+      <c r="E63">
+        <v>0</v>
       </c>
       <c r="F63">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="G63">
-        <v>0.01</v>
+        <v>0</v>
+      </c>
+      <c r="H63" t="str">
+        <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64">
-        <v>4012</v>
+        <v>3001</v>
       </c>
       <c r="B64" t="str">
         <v/>
@@ -1883,57 +2073,66 @@
       </c>
       <c r="G64">
         <v>0</v>
+      </c>
+      <c r="H64" t="str">
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65">
-        <v>9998</v>
+        <v>3333</v>
       </c>
       <c r="B65">
-        <v>0</v>
+        <v>0.71</v>
       </c>
       <c r="C65">
-        <v>0</v>
+        <v>0.41</v>
       </c>
       <c r="D65">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>0.49</v>
       </c>
       <c r="F65">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="G65">
-        <v>0</v>
+        <v>2.57</v>
+      </c>
+      <c r="H65" t="str">
+        <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66">
-        <v>13425</v>
-      </c>
-      <c r="B66">
-        <v>858.01</v>
-      </c>
-      <c r="C66">
-        <v>774.97</v>
-      </c>
-      <c r="D66">
-        <v>858.01</v>
-      </c>
-      <c r="E66">
-        <v>641.16</v>
+        <v>4011</v>
+      </c>
+      <c r="B66" t="str">
+        <v/>
+      </c>
+      <c r="C66" t="str">
+        <v/>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v/>
       </c>
       <c r="F66">
-        <v>9.67</v>
+        <v>0.01</v>
       </c>
       <c r="G66">
-        <v>3141.82</v>
+        <v>0.01</v>
+      </c>
+      <c r="H66" t="str">
+        <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="str">
-        <v/>
+      <c r="A67">
+        <v>4012</v>
       </c>
       <c r="B67" t="str">
         <v/>
@@ -1947,92 +2146,260 @@
       <c r="E67" t="str">
         <v/>
       </c>
-      <c r="F67" t="str">
-        <v/>
-      </c>
-      <c r="G67" t="str">
+      <c r="F67">
+        <v>0</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67" t="str">
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="str">
-        <v>── untagged ──</v>
-      </c>
-      <c r="B68" t="str">
-        <v/>
-      </c>
-      <c r="C68" t="str">
-        <v/>
-      </c>
-      <c r="D68" t="str">
-        <v/>
-      </c>
-      <c r="E68" t="str">
-        <v/>
-      </c>
-      <c r="F68" t="str">
-        <v/>
-      </c>
-      <c r="G68" t="str">
+      <c r="A68">
+        <v>9998</v>
+      </c>
+      <c r="B68">
+        <v>0</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+      <c r="E68">
+        <v>0</v>
+      </c>
+      <c r="F68">
+        <v>0</v>
+      </c>
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68" t="str">
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69">
+        <v>13425</v>
+      </c>
+      <c r="B69">
+        <v>858.01</v>
+      </c>
+      <c r="C69">
+        <v>774.97</v>
+      </c>
+      <c r="D69">
+        <v>858.01</v>
+      </c>
+      <c r="E69">
+        <v>641.16</v>
+      </c>
+      <c r="F69">
+        <v>9.67</v>
+      </c>
+      <c r="G69">
+        <v>3141.82</v>
+      </c>
+      <c r="H69" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v/>
+      </c>
+      <c r="B70" t="str">
+        <v/>
+      </c>
+      <c r="C70" t="str">
+        <v/>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
+      <c r="H70" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>── untagged ──</v>
+      </c>
+      <c r="B71" t="str">
+        <v/>
+      </c>
+      <c r="C71" t="str">
+        <v/>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
+      <c r="H71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
         <v>-999999</v>
       </c>
-      <c r="B69">
+      <c r="B72">
         <v>17418.88</v>
       </c>
-      <c r="C69">
+      <c r="C72">
         <v>10907.25</v>
       </c>
-      <c r="D69">
+      <c r="D72">
         <v>25305.28</v>
       </c>
-      <c r="E69">
+      <c r="E72">
         <v>18026.83</v>
       </c>
-      <c r="F69">
+      <c r="F72">
         <v>15780.23</v>
       </c>
-      <c r="G69">
+      <c r="G72">
         <v>87438.47</v>
       </c>
-    </row>
-    <row r="70">
-      <c r="A70">
+      <c r="H72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
         <v>99</v>
       </c>
-      <c r="B70">
+      <c r="B73">
         <v>1602756.97</v>
       </c>
-      <c r="C70">
+      <c r="C73">
         <v>1541979.87</v>
       </c>
-      <c r="D70">
+      <c r="D73">
         <v>1790892.59</v>
       </c>
-      <c r="E70">
+      <c r="E73">
         <v>1722310.47</v>
       </c>
-      <c r="F70">
+      <c r="F73">
         <v>1895178.54</v>
       </c>
-      <c r="G70">
+      <c r="G73">
         <v>8553118.44</v>
+      </c>
+      <c r="H73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74">
+        <v>123623963915635</v>
+      </c>
+      <c r="B74" t="str">
+        <v/>
+      </c>
+      <c r="C74" t="str">
+        <v/>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+      <c r="G74">
+        <v>0</v>
+      </c>
+      <c r="H74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75">
+        <v>90000000000000000000</v>
+      </c>
+      <c r="B75" t="str">
+        <v/>
+      </c>
+      <c r="C75" t="str">
+        <v/>
+      </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
+      <c r="F75" t="str">
+        <v/>
+      </c>
+      <c r="G75">
+        <v>0</v>
+      </c>
+      <c r="H75" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>untagged</v>
+      </c>
+      <c r="B76" t="str">
+        <v/>
+      </c>
+      <c r="C76" t="str">
+        <v/>
+      </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+      <c r="G76">
+        <v>0</v>
+      </c>
+      <c r="H76" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H76"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G69"/>
+  <dimension ref="A1:H69"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
@@ -2041,6 +2408,7 @@
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
     <col min="6" max="6" width="13.83203125" customWidth="1"/>
     <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2065,6 +2433,9 @@
       <c r="G1" t="str">
         <v>total</v>
       </c>
+      <c r="H1" t="str">
+        <v>notes</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2088,6 +2459,9 @@
       <c r="G2">
         <v>0</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -2111,6 +2485,9 @@
       <c r="G3">
         <v>0</v>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2134,6 +2511,9 @@
       <c r="G4">
         <v>62.45</v>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2157,6 +2537,9 @@
       <c r="G5">
         <v>367746.73</v>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2180,6 +2563,9 @@
       <c r="G6">
         <v>183.39</v>
       </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2203,6 +2589,9 @@
       <c r="G7">
         <v>476.01</v>
       </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2226,6 +2615,9 @@
       <c r="G8">
         <v>14506.79</v>
       </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2249,6 +2641,9 @@
       <c r="G9">
         <v>443531.96</v>
       </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -2272,6 +2667,9 @@
       <c r="G10">
         <v>38223.42</v>
       </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2295,6 +2693,9 @@
       <c r="G11">
         <v>66951.14</v>
       </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -2318,6 +2719,9 @@
       <c r="G12">
         <v>0</v>
       </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -2341,6 +2745,9 @@
       <c r="G13">
         <v>577794.63</v>
       </c>
+      <c r="H13" t="str">
+        <v>Subproxy holdings, no DR applied. Handled in Supply Side MSC.</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -2364,6 +2771,9 @@
       <c r="G14">
         <v>11597.75</v>
       </c>
+      <c r="H14" t="str">
+        <v>Spark untagged Savings, had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -2387,6 +2797,9 @@
       <c r="G15">
         <v>5643549.22</v>
       </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -2410,6 +2823,9 @@
       <c r="G16">
         <v>4.12</v>
       </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -2433,6 +2849,9 @@
       <c r="G17">
         <v>12460.39</v>
       </c>
+      <c r="H17" t="str">
+        <v>Found in Spark datasets only, no onchain events.</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -2456,6 +2875,9 @@
       <c r="G18">
         <v>0</v>
       </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -2479,6 +2901,9 @@
       <c r="G19">
         <v>0</v>
       </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -2502,6 +2927,9 @@
       <c r="G20">
         <v>0.05</v>
       </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -2525,6 +2953,9 @@
       <c r="G21">
         <v>67486.64</v>
       </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -2548,6 +2979,9 @@
       <c r="G22">
         <v>4922.33</v>
       </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -2571,6 +3005,9 @@
       <c r="G23">
         <v>36868.99</v>
       </c>
+      <c r="H23" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -2594,6 +3031,9 @@
       <c r="G24">
         <v>25603.9</v>
       </c>
+      <c r="H24" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -2617,6 +3057,9 @@
       <c r="G25">
         <v>52263.23</v>
       </c>
+      <c r="H25" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -2640,6 +3083,9 @@
       <c r="G26">
         <v>84442.43</v>
       </c>
+      <c r="H26" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -2663,6 +3109,9 @@
       <c r="G27">
         <v>9.04</v>
       </c>
+      <c r="H27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -2686,6 +3135,9 @@
       <c r="G28">
         <v>8499.05</v>
       </c>
+      <c r="H28" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -2709,6 +3161,9 @@
       <c r="G29">
         <v>0.4</v>
       </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -2732,6 +3187,9 @@
       <c r="G30">
         <v>37954.02</v>
       </c>
+      <c r="H30" t="str">
+        <v>stUSDS. Amatsu/BA applied DR in Jan./Feb. then switched to 0.1% after. s/b 0.1% always applied.</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -2755,6 +3213,9 @@
       <c r="G31">
         <v>0.1</v>
       </c>
+      <c r="H31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -2778,6 +3239,9 @@
       <c r="G32">
         <v>132.59</v>
       </c>
+      <c r="H32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -2801,6 +3265,9 @@
       <c r="G33">
         <v>177.01</v>
       </c>
+      <c r="H33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -2824,6 +3291,9 @@
       <c r="G34">
         <v>83.02</v>
       </c>
+      <c r="H34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -2847,6 +3317,9 @@
       <c r="G35">
         <v>0.64</v>
       </c>
+      <c r="H35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -2870,6 +3343,9 @@
       <c r="G36">
         <v>0</v>
       </c>
+      <c r="H36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -2893,6 +3369,9 @@
       <c r="G37">
         <v>0</v>
       </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -2916,6 +3395,9 @@
       <c r="G38">
         <v>427.02</v>
       </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -2939,6 +3421,9 @@
       <c r="G39">
         <v>14.26</v>
       </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -2962,6 +3447,9 @@
       <c r="G40">
         <v>0</v>
       </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -2985,6 +3473,9 @@
       <c r="G41">
         <v>4582.17</v>
       </c>
+      <c r="H41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -3008,6 +3499,9 @@
       <c r="G42">
         <v>0</v>
       </c>
+      <c r="H42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -3031,6 +3525,9 @@
       <c r="G43">
         <v>0</v>
       </c>
+      <c r="H43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -3054,6 +3551,9 @@
       <c r="G44">
         <v>7604.96</v>
       </c>
+      <c r="H44" t="str">
+        <v>Feb. and Mar. had no DR by Amatsu.</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -3077,6 +3577,9 @@
       <c r="G45">
         <v>96262.58</v>
       </c>
+      <c r="H45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -3100,6 +3603,9 @@
       <c r="G46">
         <v>0.04</v>
       </c>
+      <c r="H46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -3123,6 +3629,9 @@
       <c r="G47">
         <v>64561.56</v>
       </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -3146,6 +3655,9 @@
       <c r="G48">
         <v>0</v>
       </c>
+      <c r="H48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -3169,6 +3681,9 @@
       <c r="G49">
         <v>1378.16</v>
       </c>
+      <c r="H49" t="str">
+        <v>Amatsu included DR for sUSDC, sUSDS, SKY, while onchain, only events for SKY can be found. unknown which balances or events to use for sUSDC and sUSDS.</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -3192,6 +3707,9 @@
       <c r="G50">
         <v>593.4</v>
       </c>
+      <c r="H50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -3215,6 +3733,9 @@
       <c r="G51">
         <v>0</v>
       </c>
+      <c r="H51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -3238,6 +3759,9 @@
       <c r="G52">
         <v>8550.23</v>
       </c>
+      <c r="H52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -3261,6 +3785,9 @@
       <c r="G53">
         <v>291311.65</v>
       </c>
+      <c r="H53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -3284,6 +3811,9 @@
       <c r="G54">
         <v>0</v>
       </c>
+      <c r="H54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -3307,6 +3837,9 @@
       <c r="G55">
         <v>25404.85</v>
       </c>
+      <c r="H55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -3330,6 +3863,9 @@
       <c r="G56">
         <v>12035.78</v>
       </c>
+      <c r="H56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -3353,6 +3889,9 @@
       <c r="G57">
         <v>25.43</v>
       </c>
+      <c r="H57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -3376,6 +3915,9 @@
       <c r="G58">
         <v>0</v>
       </c>
+      <c r="H58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -3399,6 +3941,9 @@
       <c r="G59">
         <v>0</v>
       </c>
+      <c r="H59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -3422,6 +3967,9 @@
       <c r="G60">
         <v>2.57</v>
       </c>
+      <c r="H60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -3445,6 +3993,9 @@
       <c r="G61">
         <v>0.01</v>
       </c>
+      <c r="H61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -3468,6 +4019,9 @@
       <c r="G62">
         <v>0</v>
       </c>
+      <c r="H62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -3491,6 +4045,9 @@
       <c r="G63">
         <v>0</v>
       </c>
+      <c r="H63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -3514,6 +4071,9 @@
       <c r="G64">
         <v>3141.82</v>
       </c>
+      <c r="H64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3535,6 +4095,9 @@
         <v/>
       </c>
       <c r="G65" t="str">
+        <v/>
+      </c>
+      <c r="H65" t="str">
         <v/>
       </c>
     </row>
@@ -3560,6 +4123,9 @@
       <c r="G66" t="str">
         <v/>
       </c>
+      <c r="H66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -3583,6 +4149,9 @@
       <c r="G67">
         <v>7260378.37</v>
       </c>
+      <c r="H67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -3606,6 +4175,9 @@
       <c r="G68">
         <v>0.02</v>
       </c>
+      <c r="H68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -3629,23 +4201,27 @@
       <c r="G69">
         <v>0.07</v>
       </c>
+      <c r="H69" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H69"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:F43"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.83203125" customWidth="1"/>
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="55.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3664,6 +4240,9 @@
       <c r="E1" t="str">
         <v>total</v>
       </c>
+      <c r="F1" t="str">
+        <v>notes</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -3681,6 +4260,9 @@
       <c r="E2">
         <v>53206</v>
       </c>
+      <c r="F2" t="str">
+        <v>Spark untagged Savings, had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -3698,6 +4280,9 @@
       <c r="E3">
         <v>3602072.3</v>
       </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -3715,6 +4300,9 @@
       <c r="E4">
         <v>4.4</v>
       </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -3732,6 +4320,9 @@
       <c r="E5">
         <v>0</v>
       </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -3749,6 +4340,9 @@
       <c r="E6">
         <v>0</v>
       </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -3766,6 +4360,9 @@
       <c r="E7">
         <v>0</v>
       </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8">
@@ -3783,6 +4380,9 @@
       <c r="E8">
         <v>45724.8</v>
       </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9">
@@ -3800,6 +4400,9 @@
       <c r="E9">
         <v>5624.6</v>
       </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10">
@@ -3817,6 +4420,9 @@
       <c r="E10">
         <v>18219.7</v>
       </c>
+      <c r="F10" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11">
@@ -3834,6 +4440,9 @@
       <c r="E11">
         <v>48038.5</v>
       </c>
+      <c r="F11" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12">
@@ -3851,6 +4460,9 @@
       <c r="E12">
         <v>39358</v>
       </c>
+      <c r="F12" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -3868,6 +4480,9 @@
       <c r="E13">
         <v>146684.5</v>
       </c>
+      <c r="F13" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -3885,6 +4500,9 @@
       <c r="E14">
         <v>14</v>
       </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -3902,6 +4520,9 @@
       <c r="E15">
         <v>13163</v>
       </c>
+      <c r="F15" t="str">
+        <v>Had boosted DR applied by Amatsu.</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -3919,6 +4540,9 @@
       <c r="E16">
         <v>0.5</v>
       </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -3936,6 +4560,9 @@
       <c r="E17">
         <v>70977.9</v>
       </c>
+      <c r="F17" t="str">
+        <v>stUSDS. Amatsu/BA applied DR in Jan./Feb. then switched to 0.1% after. s/b 0.1% always applied.</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -3953,6 +4580,9 @@
       <c r="E18">
         <v>0</v>
       </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -3970,6 +4600,9 @@
       <c r="E19">
         <v>19.6</v>
       </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -3987,6 +4620,9 @@
       <c r="E20">
         <v>243.8</v>
       </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -4004,6 +4640,9 @@
       <c r="E21">
         <v>45.6</v>
       </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -4021,6 +4660,9 @@
       <c r="E22">
         <v>0.5</v>
       </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -4038,6 +4680,9 @@
       <c r="E23">
         <v>216.5</v>
       </c>
+      <c r="F23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -4055,6 +4700,9 @@
       <c r="E24">
         <v>0</v>
       </c>
+      <c r="F24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -4072,6 +4720,9 @@
       <c r="E25">
         <v>0</v>
       </c>
+      <c r="F25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -4089,6 +4740,9 @@
       <c r="E26">
         <v>0</v>
       </c>
+      <c r="F26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -4106,6 +4760,9 @@
       <c r="E27">
         <v>2255</v>
       </c>
+      <c r="F27" t="str">
+        <v>Feb. and Mar. had no DR by Amatsu.</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -4123,6 +4780,9 @@
       <c r="E28">
         <v>34121.3</v>
       </c>
+      <c r="F28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -4140,6 +4800,9 @@
       <c r="E29">
         <v>178305.2</v>
       </c>
+      <c r="F29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -4157,6 +4820,9 @@
       <c r="E30">
         <v>1024.6</v>
       </c>
+      <c r="F30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -4174,6 +4840,9 @@
       <c r="E31">
         <v>39681.5</v>
       </c>
+      <c r="F31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -4191,6 +4860,9 @@
       <c r="E32">
         <v>0</v>
       </c>
+      <c r="F32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -4208,6 +4880,9 @@
       <c r="E33">
         <v>12676.1</v>
       </c>
+      <c r="F33" t="str">
+        <v>Amatsu included DR for sUSDC, sUSDS, SKY, while onchain, only events for SKY can be found. unknown which balances or events to use for sUSDC and sUSDS.</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -4225,6 +4900,9 @@
       <c r="E34">
         <v>1256</v>
       </c>
+      <c r="F34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -4242,6 +4920,9 @@
       <c r="E35">
         <v>0</v>
       </c>
+      <c r="F35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -4259,6 +4940,9 @@
       <c r="E36">
         <v>0</v>
       </c>
+      <c r="F36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -4276,6 +4960,9 @@
       <c r="E37">
         <v>174513</v>
       </c>
+      <c r="F37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -4293,6 +4980,9 @@
       <c r="E38">
         <v>0</v>
       </c>
+      <c r="F38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -4310,6 +5000,9 @@
       <c r="E39">
         <v>17129.9</v>
       </c>
+      <c r="F39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -4327,6 +5020,9 @@
       <c r="E40">
         <v>0</v>
       </c>
+      <c r="F40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -4342,6 +5038,9 @@
         <v/>
       </c>
       <c r="E41" t="str">
+        <v/>
+      </c>
+      <c r="F41" t="str">
         <v/>
       </c>
     </row>
@@ -4361,6 +5060,9 @@
       <c r="E42" t="str">
         <v/>
       </c>
+      <c r="F42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -4378,10 +5080,13 @@
       <c r="E43">
         <v>4813357.6</v>
       </c>
+      <c r="F43" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F43"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4551,7 +5256,7 @@
         <v>0 (USDS-CLE)</v>
       </c>
       <c r="B6" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -4572,7 +5277,7 @@
         <v>1786.39</v>
       </c>
       <c r="I6" t="str">
-        <v>Chronicle farm — not tracked by Spark.</v>
+        <v>Chronicle farm — not tracked by Spark/BA.</v>
       </c>
     </row>
     <row r="7">
@@ -4696,7 +5401,7 @@
         <v>1 (USDS-CLE)</v>
       </c>
       <c r="B11" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C11">
         <v>5139.57</v>
@@ -4717,7 +5422,7 @@
         <v>29341.39</v>
       </c>
       <c r="I11" t="str">
-        <v>Chronicle farm — not tracked by Spark.</v>
+        <v>Chronicle farm — not tracked by Spark/BA.</v>
       </c>
     </row>
     <row r="12">
@@ -4812,7 +5517,7 @@
         <v>10</v>
       </c>
       <c r="B15" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -4841,7 +5546,7 @@
         <v>100</v>
       </c>
       <c r="B16" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -4920,7 +5625,7 @@
         <v>-1575.56</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>Spark untagged Savings, had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="19">
@@ -5181,7 +5886,7 @@
         <v>-2893.69</v>
       </c>
       <c r="I27" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="28">
@@ -5210,7 +5915,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="29">
@@ -5239,7 +5944,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="30">
@@ -5268,7 +5973,7 @@
         <v>0</v>
       </c>
       <c r="I30" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="31">
@@ -5326,7 +6031,7 @@
         <v>0</v>
       </c>
       <c r="I32" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="33">
@@ -5384,7 +6089,7 @@
         <v>0</v>
       </c>
       <c r="I34" t="str">
-        <v/>
+        <v>stUSDS. Amatsu/BA applied DR in Jan./Feb. then switched to 0.1% after. s/b 0.1% always applied.</v>
       </c>
     </row>
     <row r="35">
@@ -5790,7 +6495,7 @@
         <v>253.28</v>
       </c>
       <c r="I48" t="str">
-        <v/>
+        <v>Feb. and Mar. had no DR by Amatsu.</v>
       </c>
     </row>
     <row r="49">
@@ -5935,7 +6640,7 @@
         <v>0</v>
       </c>
       <c r="I53" t="str">
-        <v/>
+        <v>Amatsu included DR for sUSDC, sUSDS, SKY, while onchain, only events for SKY can be found. unknown which balances or events to use for sUSDC and sUSDS.</v>
       </c>
     </row>
     <row r="54">
@@ -6436,7 +7141,7 @@
         <v>-999999</v>
       </c>
       <c r="B71" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C71">
         <v>17418.88</v>
@@ -6595,7 +7300,7 @@
         <v>0 (spUSDC)</v>
       </c>
       <c r="B2" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -6618,7 +7323,7 @@
         <v>0 (stUSDS)</v>
       </c>
       <c r="B3" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -6641,7 +7346,7 @@
         <v>0 (sUSDC)</v>
       </c>
       <c r="B4" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C4">
         <v>14.3</v>
@@ -6664,7 +7369,7 @@
         <v>0 (sUSDS)</v>
       </c>
       <c r="B5" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C5">
         <v>79746.04</v>
@@ -6687,7 +7392,7 @@
         <v>0 (USDS-CLE)</v>
       </c>
       <c r="B6" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -6702,7 +7407,7 @@
         <v>324.57</v>
       </c>
       <c r="G6" t="str">
-        <v>Chronicle farm — not tracked by Spark.</v>
+        <v>Chronicle farm — not tracked by Spark/BA.</v>
       </c>
     </row>
     <row r="7">
@@ -6710,7 +7415,7 @@
         <v>0 (USDS-SKY)</v>
       </c>
       <c r="B7" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C7">
         <v>93.87</v>
@@ -6733,7 +7438,7 @@
         <v>0 (USDS-SPK)</v>
       </c>
       <c r="B8" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -6756,7 +7461,7 @@
         <v>1 (stUSDS)</v>
       </c>
       <c r="B9" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C9">
         <v>1800.55</v>
@@ -6779,7 +7484,7 @@
         <v>1 (sUSDS)</v>
       </c>
       <c r="B10" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C10">
         <v>81433.39</v>
@@ -6802,7 +7507,7 @@
         <v>1 (USDS-CLE)</v>
       </c>
       <c r="B11" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C11">
         <v>5139.57</v>
@@ -6817,7 +7522,7 @@
         <v>15593.34</v>
       </c>
       <c r="G11" t="str">
-        <v>Chronicle farm — not tracked by Spark.</v>
+        <v>Chronicle farm — not tracked by Spark/BA.</v>
       </c>
     </row>
     <row r="12">
@@ -6825,7 +7530,7 @@
         <v>1 (USDS-SKY)</v>
       </c>
       <c r="B12" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C12">
         <v>26939.34</v>
@@ -6848,7 +7553,7 @@
         <v>1 (USDS-SPK)</v>
       </c>
       <c r="B13" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C13">
         <v>14315.55</v>
@@ -6871,7 +7576,7 @@
         <v>2</v>
       </c>
       <c r="B14" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -6894,7 +7599,7 @@
         <v>10</v>
       </c>
       <c r="B15" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -6917,7 +7622,7 @@
         <v>100</v>
       </c>
       <c r="B16" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -6955,7 +7660,7 @@
         <v>-45362.23</v>
       </c>
       <c r="G17" t="str">
-        <v/>
+        <v>Spark untagged Savings, had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="18">
@@ -7139,7 +7844,7 @@
         <v>-10434.71</v>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="26">
@@ -7162,7 +7867,7 @@
         <v>-28087.56</v>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="27">
@@ -7185,7 +7890,7 @@
         <v>-22460.06</v>
       </c>
       <c r="G27" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="28">
@@ -7208,7 +7913,7 @@
         <v>-87916.08</v>
       </c>
       <c r="G28" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="29">
@@ -7254,7 +7959,7 @@
         <v>-7889.26</v>
       </c>
       <c r="G30" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="31">
@@ -7300,7 +8005,7 @@
         <v>-52262.69</v>
       </c>
       <c r="G32" t="str">
-        <v/>
+        <v>stUSDS. Amatsu/BA applied DR in Jan./Feb. then switched to 0.1% after. s/b 0.1% always applied.</v>
       </c>
     </row>
     <row r="33">
@@ -7423,7 +8128,7 @@
         <v>206</v>
       </c>
       <c r="B38" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C38">
         <v>0</v>
@@ -7446,7 +8151,7 @@
         <v>214</v>
       </c>
       <c r="B39" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -7515,7 +8220,7 @@
         <v>223</v>
       </c>
       <c r="B42" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C42">
         <v>0</v>
@@ -7538,7 +8243,7 @@
         <v>224</v>
       </c>
       <c r="B43" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C43">
         <v>0</v>
@@ -7622,7 +8327,7 @@
         <v>3256.73</v>
       </c>
       <c r="G46" t="str">
-        <v/>
+        <v>Feb. and Mar. had no DR by Amatsu.</v>
       </c>
     </row>
     <row r="47">
@@ -7760,7 +8465,7 @@
         <v>-11298.53</v>
       </c>
       <c r="G52" t="str">
-        <v/>
+        <v>Amatsu included DR for sUSDC, sUSDS, SKY, while onchain, only events for SKY can be found. unknown which balances or events to use for sUSDC and sUSDS.</v>
       </c>
     </row>
     <row r="53">
@@ -7906,7 +8611,7 @@
         <v>2008</v>
       </c>
       <c r="B59" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C59">
         <v>0</v>
@@ -7952,7 +8657,7 @@
         <v>3000</v>
       </c>
       <c r="B61" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -7975,7 +8680,7 @@
         <v>3001</v>
       </c>
       <c r="B62" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -7998,7 +8703,7 @@
         <v>3333</v>
       </c>
       <c r="B63" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C63">
         <v>0.71</v>
@@ -8021,7 +8726,7 @@
         <v>4011</v>
       </c>
       <c r="B64" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -8044,7 +8749,7 @@
         <v>4012</v>
       </c>
       <c r="B65" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -8067,7 +8772,7 @@
         <v>9998</v>
       </c>
       <c r="B66" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -8090,7 +8795,7 @@
         <v>13425</v>
       </c>
       <c r="B67" t="str">
-        <v>ours only</v>
+        <v>soter only</v>
       </c>
       <c r="C67">
         <v>858.01</v>
@@ -8516,7 +9221,7 @@
         <v>-44356.89</v>
       </c>
       <c r="G14" t="str">
-        <v/>
+        <v>Spark untagged Savings, had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="15">
@@ -8723,7 +9428,7 @@
         <v>-7979.33</v>
       </c>
       <c r="G23" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="24">
@@ -8746,7 +9451,7 @@
         <v>-28087.56</v>
       </c>
       <c r="G24" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="25">
@@ -8769,7 +9474,7 @@
         <v>-22460.06</v>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="26">
@@ -8792,7 +9497,7 @@
         <v>-87916.08</v>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="27">
@@ -8838,7 +9543,7 @@
         <v>-7889.26</v>
       </c>
       <c r="G28" t="str">
-        <v/>
+        <v>Had boosted DR applied by Amatsu.</v>
       </c>
     </row>
     <row r="29">
@@ -8884,7 +9589,7 @@
         <v>-52262.69</v>
       </c>
       <c r="G30" t="str">
-        <v/>
+        <v>stUSDS. Amatsu/BA applied DR in Jan./Feb. then switched to 0.1% after. s/b 0.1% always applied.</v>
       </c>
     </row>
     <row r="31">
@@ -9206,7 +9911,7 @@
         <v>3089.33</v>
       </c>
       <c r="G44" t="str">
-        <v/>
+        <v>Feb. and Mar. had no DR by Amatsu.</v>
       </c>
     </row>
     <row r="45">
@@ -9344,7 +10049,7 @@
         <v>-11298.53</v>
       </c>
       <c r="G50" t="str">
-        <v/>
+        <v>Amatsu included DR for sUSDC, sUSDS, SKY, while onchain, only events for SKY can be found. unknown which balances or events to use for sUSDC and sUSDS.</v>
       </c>
     </row>
     <row r="51">

</xml_diff>